<commit_message>
new segment and feedback updated
</commit_message>
<xml_diff>
--- a/AGMC_Portal_Screens_Menus_and_APIs_Documentation.xlsx
+++ b/AGMC_Portal_Screens_Menus_and_APIs_Documentation.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="7500"/>
+    <workbookView windowWidth="20490" windowHeight="7500" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Executive Summary" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="681" uniqueCount="385">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="651" uniqueCount="356">
   <si>
     <t>AGMC CUSTOMER EXPERIENCE &amp; OPERATIONS PORTAL</t>
   </si>
@@ -56,7 +56,7 @@
     <t>Direct Keyloop &amp; Desktop Interface</t>
   </si>
   <si>
-    <t>Dealer-local (+04:00)</t>
+    <t xml:space="preserve">Dealer-local </t>
   </si>
   <si>
     <t>Keyloop Group Brands</t>
@@ -101,7 +101,7 @@
     <t>Sales Portal</t>
   </si>
   <si>
-    <t>Overview, New Lead, Enquiries, Test Drive, Vehicle Orders, Customer Segments, After-Sales</t>
+    <t>Overview, New Lead, Enquiries, Test Drive, Vehicle Orders, Customer Segments, After-Sales &amp; Follow up</t>
   </si>
   <si>
     <t>Service &amp; Booking</t>
@@ -134,9 +134,6 @@
     <t>Submenu / Tab Name</t>
   </si>
   <si>
-    <t>Component File</t>
-  </si>
-  <si>
     <t>Key Functional Features &amp; User Workflow</t>
   </si>
   <si>
@@ -153,9 +150,6 @@
   </si>
   <si>
     <t>Customer 360 &amp; Search</t>
-  </si>
-  <si>
-    <t>LeftSidebar.jsx / CustomerContext.jsx</t>
   </si>
   <si>
     <t>Mobile lookup (Caller ID discovery), Customer selector dropdown for multiple accounts, VIP status, contact details, branch, consents, verification badge, and risk level card</t>
@@ -171,9 +165,6 @@
     <t>Customer Vehicles &amp; Activity</t>
   </si>
   <si>
-    <t>RightSidebar.jsx / ServiceCustomerVehicleCard.jsx</t>
-  </si>
-  <si>
     <t>Customer vehicle carousel/selector (VIN, brand, model, colour, odometer, warranty, service contract) + Real-time complaint timeline with priority filters</t>
   </si>
   <si>
@@ -188,9 +179,6 @@
     <t>Overview</t>
   </si>
   <si>
-    <t>OverviewView.jsx</t>
-  </si>
-  <si>
     <t>High-level summary of customer complaints, open vs closed tickets breakdown, ticket volume status, quick escalation alerts</t>
   </si>
   <si>
@@ -201,9 +189,6 @@
     <t>Create Complaint</t>
   </si>
   <si>
-    <t>CreateComplaintView.jsx</t>
-  </si>
-  <si>
     <t>Form to lodge new customer complaints with category, branch, priority, detailed description, auto-agent identification</t>
   </si>
   <si>
@@ -213,9 +198,6 @@
     <t>Open Complaints</t>
   </si>
   <si>
-    <t>OpenComplaintsView.jsx</t>
-  </si>
-  <si>
     <t>Lists all open active complaint tickets for the selected customer, origin badge (KEYLOOP vs DESKTOP), category, and creation date</t>
   </si>
   <si>
@@ -223,9 +205,6 @@
   </si>
   <si>
     <t>Recovery Actions</t>
-  </si>
-  <si>
-    <t>RecoveryActionsView.jsx</t>
   </si>
   <si>
     <t>Select complaint ticket, view existing recovery action, create new recovery action, update recovery action against actionId, cancel action. Zero dummy data.</t>
@@ -241,9 +220,6 @@
     <t>Assign Complaint</t>
   </si>
   <si>
-    <t>AssignComplaintView.jsx</t>
-  </si>
-  <si>
     <t>Real-time assignment status badge (ASSIGNED vs UNASSIGNED), ticket selector, allocation form to assign/reassign to agent or unassign ticket. Zero dummy fields.</t>
   </si>
   <si>
@@ -255,9 +231,6 @@
     <t>Resolve Complaint</t>
   </si>
   <si>
-    <t>ResolveComplaintView.jsx</t>
-  </si>
-  <si>
     <t>Live resolution status (OPEN vs RESOLVED), formal closure with resolution code (Apology, Goodwill Gesture, etc.) and resolution notes. Locks form when resolved.</t>
   </si>
   <si>
@@ -267,9 +240,6 @@
   </si>
   <si>
     <t>/sales</t>
-  </si>
-  <si>
-    <t>SalesOverviewView.jsx</t>
   </si>
   <si>
     <t>Comprehensive 360 sales snapshot: Active vehicles, finance agreements, insurance policies, trade-in history, sales summary</t>
@@ -286,9 +256,6 @@
     <t>New Lead</t>
   </si>
   <si>
-    <t>SalesNewLeadView.jsx</t>
-  </si>
-  <si>
     <t>Lead capture form: customer contact info, vehicle interest, test drive request, purchase timeline, escalation to complaint creation</t>
   </si>
   <si>
@@ -301,9 +268,6 @@
     <t>Enquiries</t>
   </si>
   <si>
-    <t>SalesEnquiriesView.jsx</t>
-  </si>
-  <si>
     <t>Keyloop enquiries list: WON/LOST badges, order/invoice details, branch &amp; sales executive, expandable record with enrolled journeys (J01 showroom, J03 delivery)</t>
   </si>
   <si>
@@ -316,9 +280,6 @@
     <t>Test Drive</t>
   </si>
   <si>
-    <t>SalesTestDriveView.jsx</t>
-  </si>
-  <si>
     <t>Test drive booking panel, real-time available time-slot lookup by branch/date/model, active booking history, advisor assignment</t>
   </si>
   <si>
@@ -329,9 +290,6 @@
   </si>
   <si>
     <t>Vehicle Orders</t>
-  </si>
-  <si>
-    <t>SalesVehicleOrdersView.jsx</t>
   </si>
   <si>
     <t>Tracking vehicle orders &amp; delivery pipeline: Production stages, shipment updates, RTA vehicle registration progress, readiness for handover checklist</t>
@@ -349,9 +307,6 @@
     <t>Customer Segments</t>
   </si>
   <si>
-    <t>SalesSegmentsView.jsx</t>
-  </si>
-  <si>
     <t>Customer segmentation profiling: VIP tier, loyalty status, high-net-worth segment classification, upgrade propensity</t>
   </si>
   <si>
@@ -359,9 +314,6 @@
   </si>
   <si>
     <t>After-Sales &amp; Follow Up</t>
-  </si>
-  <si>
-    <t>SalesAfterSalesView.jsx</t>
   </si>
   <si>
     <t>After-sales relationship tracking: Vehicle delivery follow-up, service booking history, customer contact logs, next action reminders</t>
@@ -373,9 +325,6 @@
   </si>
   <si>
     <t>/service</t>
-  </si>
-  <si>
-    <t>ServiceOverviewView.jsx</t>
   </si>
   <si>
     <t>Live vehicle health dashboard: Next service due date &amp; km, last service history, warranty package status, active service inclusive contract</t>
@@ -388,9 +337,6 @@
   </si>
   <si>
     <t>Book Service</t>
-  </si>
-  <si>
-    <t>ServiceBookingMainPanel.jsx</t>
   </si>
   <si>
     <t>Workshop booking workbench: Request service appointment, package eligibility check, WIP booking creation, booking confirmation slip, reminder dispatch, recommended packages</t>
@@ -409,9 +355,6 @@
     <t>Open Bookings</t>
   </si>
   <si>
-    <t>ServiceOpenBookingsView.jsx</t>
-  </si>
-  <si>
     <t>Active workshop jobs: List open appointments, assigned service advisor, WIP number, scheduled time, service job description</t>
   </si>
   <si>
@@ -421,9 +364,6 @@
     <t>Service History</t>
   </si>
   <si>
-    <t>ServiceHistoryView.jsx</t>
-  </si>
-  <si>
     <t>Historical vehicle maintenance timeline: Previous work orders, invoice numbers, service date, mileage recorded, operations performed</t>
   </si>
   <si>
@@ -433,9 +373,6 @@
     <t>Warranty Claims</t>
   </si>
   <si>
-    <t>ServiceWarrantyClaimsView.jsx</t>
-  </si>
-  <si>
     <t>Historical &amp; active manufacturer warranty claims: Claim ID, defect code, claimed parts, status (APPROVED / REJECTED / PENDING)</t>
   </si>
   <si>
@@ -445,9 +382,6 @@
     <t>Service Feedback</t>
   </si>
   <si>
-    <t>ServiceFeedbackView.jsx</t>
-  </si>
-  <si>
     <t>Post-service customer feedback ratings, survey remarks, workshop satisfaction scores</t>
   </si>
   <si>
@@ -461,9 +395,6 @@
   </si>
   <si>
     <t>Overview / All Tabs</t>
-  </si>
-  <si>
-    <t>FeedbackOverviewView.jsx</t>
   </si>
   <si>
     <t>Customer Feedback Hub: CSI aggregate scores, actual customer survey responses, historical feedback logs, submit new feedback record</t>
@@ -483,24 +414,6 @@
   <si>
     <t>GET /api/v1/lost-sales/reasons?group={g}&amp;branch={b}
 GET /api/v1/lost-sales?group={g}&amp;customerNumber={c}</t>
-  </si>
-  <si>
-    <t>IMEI Tracker</t>
-  </si>
-  <si>
-    <t>/tracker</t>
-  </si>
-  <si>
-    <t>Live GPS Tracking</t>
-  </si>
-  <si>
-    <t>IMEITrackerPage.jsx</t>
-  </si>
-  <si>
-    <t>Live telematics tracking: Search by 15-digit IMEI, interactive Leaflet map with pulsing pin, coordinates, battery level, online/offline status, recent search history</t>
-  </si>
-  <si>
-    <t>POST http://localhost:3001/api/devices/track</t>
   </si>
   <si>
     <t>Profile Component / Panel</t>
@@ -1248,7 +1161,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="32">
+  <fonts count="31">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1324,13 +1237,6 @@
       <color rgb="FF555555"/>
       <name val="Calibri"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <u/>
@@ -1843,148 +1749,148 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="12" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="12" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="12" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="12" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="12" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="12" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -2442,7 +2348,7 @@
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="32" customWidth="1"/>
-    <col min="3" max="3" width="55" customWidth="1"/>
+    <col min="3" max="3" width="89.5714285714286" customWidth="1"/>
     <col min="4" max="4" width="25" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2583,20 +2489,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H25"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="7"/>
+  <dimension ref="A1:G24"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="6"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
     <col min="4" max="4" width="24" customWidth="1"/>
-    <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="45" customWidth="1"/>
-    <col min="7" max="7" width="48" customWidth="1"/>
-    <col min="8" max="8" width="10" customWidth="1"/>
+    <col min="5" max="5" width="45" customWidth="1"/>
+    <col min="6" max="6" width="48" customWidth="1"/>
+    <col min="7" max="7" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:8">
+    <row r="1" ht="30" customHeight="1" spans="1:7">
       <c r="A1" s="1" t="s">
         <v>30</v>
       </c>
@@ -2618,63 +2523,54 @@
       <c r="G1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="2" ht="36" customHeight="1" spans="1:8">
+    </row>
+    <row r="2" ht="36" customHeight="1" spans="1:7">
       <c r="A2" s="6">
         <v>1</v>
       </c>
       <c r="B2" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="F2" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="H2" s="16">
+      <c r="G2" s="16">
         <v>5</v>
       </c>
     </row>
-    <row r="3" ht="36" customHeight="1" spans="1:8">
+    <row r="3" ht="36" customHeight="1" spans="1:7">
       <c r="A3" s="10">
         <v>2</v>
       </c>
       <c r="B3" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="C3" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="C3" s="8" t="s">
-        <v>39</v>
-      </c>
       <c r="D3" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="F3" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="E3" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="F3" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="G3" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="H3" s="17">
+      <c r="G3" s="17">
         <v>3</v>
       </c>
     </row>
-    <row r="4" ht="36" customHeight="1" spans="1:8">
+    <row r="4" ht="36" customHeight="1" spans="1:7">
       <c r="A4" s="6">
         <v>3</v>
       </c>
@@ -2682,25 +2578,22 @@
         <v>19</v>
       </c>
       <c r="C4" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="D4" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="H4" s="16">
+      <c r="G4" s="16">
         <v>2</v>
       </c>
     </row>
-    <row r="5" ht="36" customHeight="1" spans="1:8">
+    <row r="5" ht="36" customHeight="1" spans="1:7">
       <c r="A5" s="10">
         <v>4</v>
       </c>
@@ -2708,25 +2601,22 @@
         <v>19</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="G5" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="H5" s="17">
+        <v>51</v>
+      </c>
+      <c r="G5" s="17">
         <v>1</v>
       </c>
     </row>
-    <row r="6" ht="36" customHeight="1" spans="1:8">
+    <row r="6" ht="36" customHeight="1" spans="1:7">
       <c r="A6" s="6">
         <v>5</v>
       </c>
@@ -2734,25 +2624,22 @@
         <v>19</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="H6" s="16">
+        <v>54</v>
+      </c>
+      <c r="G6" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="7" ht="36" customHeight="1" spans="1:8">
+    <row r="7" ht="36" customHeight="1" spans="1:7">
       <c r="A7" s="10">
         <v>6</v>
       </c>
@@ -2760,25 +2647,22 @@
         <v>19</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="G7" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="H7" s="17">
+        <v>57</v>
+      </c>
+      <c r="G7" s="17">
         <v>5</v>
       </c>
     </row>
-    <row r="8" ht="36" customHeight="1" spans="1:8">
+    <row r="8" ht="36" customHeight="1" spans="1:7">
       <c r="A8" s="6">
         <v>7</v>
       </c>
@@ -2786,25 +2670,22 @@
         <v>19</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="H8" s="16">
+        <v>60</v>
+      </c>
+      <c r="G8" s="16">
         <v>3</v>
       </c>
     </row>
-    <row r="9" ht="36" customHeight="1" spans="1:8">
+    <row r="9" ht="36" customHeight="1" spans="1:7">
       <c r="A9" s="10">
         <v>8</v>
       </c>
@@ -2812,25 +2693,22 @@
         <v>19</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="G9" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="H9" s="17">
+        <v>63</v>
+      </c>
+      <c r="G9" s="17">
         <v>3</v>
       </c>
     </row>
-    <row r="10" ht="36" customHeight="1" spans="1:8">
+    <row r="10" ht="36" customHeight="1" spans="1:7">
       <c r="A10" s="6">
         <v>9</v>
       </c>
@@ -2838,25 +2716,22 @@
         <v>22</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="H10" s="16">
+        <v>66</v>
+      </c>
+      <c r="G10" s="16">
         <v>6</v>
       </c>
     </row>
-    <row r="11" ht="36" customHeight="1" spans="1:8">
+    <row r="11" ht="36" customHeight="1" spans="1:7">
       <c r="A11" s="10">
         <v>10</v>
       </c>
@@ -2864,25 +2739,22 @@
         <v>22</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="G11" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="H11" s="17">
+        <v>69</v>
+      </c>
+      <c r="G11" s="17">
         <v>4</v>
       </c>
     </row>
-    <row r="12" ht="36" customHeight="1" spans="1:8">
+    <row r="12" ht="36" customHeight="1" spans="1:7">
       <c r="A12" s="6">
         <v>11</v>
       </c>
@@ -2890,25 +2762,22 @@
         <v>22</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>81</v>
+        <v>70</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="H12" s="16">
+        <v>72</v>
+      </c>
+      <c r="G12" s="16">
         <v>4</v>
       </c>
     </row>
-    <row r="13" ht="36" customHeight="1" spans="1:8">
+    <row r="13" ht="36" customHeight="1" spans="1:7">
       <c r="A13" s="10">
         <v>12</v>
       </c>
@@ -2916,25 +2785,22 @@
         <v>22</v>
       </c>
       <c r="C13" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="D13" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="D13" s="8" t="s">
-        <v>85</v>
-      </c>
       <c r="E13" s="8" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="G13" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="H13" s="17">
+        <v>75</v>
+      </c>
+      <c r="G13" s="17">
         <v>4</v>
       </c>
     </row>
-    <row r="14" ht="36" customHeight="1" spans="1:8">
+    <row r="14" ht="36" customHeight="1" spans="1:7">
       <c r="A14" s="6">
         <v>13</v>
       </c>
@@ -2942,25 +2808,22 @@
         <v>22</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="H14" s="16">
+        <v>78</v>
+      </c>
+      <c r="G14" s="16">
         <v>7</v>
       </c>
     </row>
-    <row r="15" ht="36" customHeight="1" spans="1:8">
+    <row r="15" ht="36" customHeight="1" spans="1:7">
       <c r="A15" s="10">
         <v>14</v>
       </c>
@@ -2968,25 +2831,22 @@
         <v>22</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>93</v>
+        <v>79</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="G15" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="H15" s="17">
+        <v>81</v>
+      </c>
+      <c r="G15" s="17">
         <v>1</v>
       </c>
     </row>
-    <row r="16" ht="36" customHeight="1" spans="1:8">
+    <row r="16" ht="36" customHeight="1" spans="1:7">
       <c r="A16" s="6">
         <v>15</v>
       </c>
@@ -2994,25 +2854,22 @@
         <v>22</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>97</v>
+        <v>82</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>98</v>
+        <v>83</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="G16" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="H16" s="16">
+        <v>84</v>
+      </c>
+      <c r="G16" s="16">
         <v>3</v>
       </c>
     </row>
-    <row r="17" ht="36" customHeight="1" spans="1:8">
+    <row r="17" ht="36" customHeight="1" spans="1:7">
       <c r="A17" s="10">
         <v>16</v>
       </c>
@@ -3020,25 +2877,22 @@
         <v>24</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="G17" s="8" t="s">
-        <v>104</v>
-      </c>
-      <c r="H17" s="17">
+        <v>87</v>
+      </c>
+      <c r="G17" s="17">
         <v>4</v>
       </c>
     </row>
-    <row r="18" ht="36" customHeight="1" spans="1:8">
+    <row r="18" ht="36" customHeight="1" spans="1:7">
       <c r="A18" s="6">
         <v>17</v>
       </c>
@@ -3046,25 +2900,22 @@
         <v>24</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>105</v>
+        <v>88</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>106</v>
+        <v>89</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="H18" s="16">
+        <v>90</v>
+      </c>
+      <c r="G18" s="16">
         <v>8</v>
       </c>
     </row>
-    <row r="19" ht="36" customHeight="1" spans="1:8">
+    <row r="19" ht="36" customHeight="1" spans="1:7">
       <c r="A19" s="10">
         <v>18</v>
       </c>
@@ -3072,25 +2923,22 @@
         <v>24</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>109</v>
+        <v>91</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>110</v>
+        <v>92</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>111</v>
-      </c>
-      <c r="G19" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="H19" s="17">
+        <v>93</v>
+      </c>
+      <c r="G19" s="17">
         <v>1</v>
       </c>
     </row>
-    <row r="20" ht="36" customHeight="1" spans="1:8">
+    <row r="20" ht="36" customHeight="1" spans="1:7">
       <c r="A20" s="6">
         <v>19</v>
       </c>
@@ -3098,25 +2946,22 @@
         <v>24</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>114</v>
+        <v>95</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="G20" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="H20" s="16">
+        <v>96</v>
+      </c>
+      <c r="G20" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="21" ht="36" customHeight="1" spans="1:8">
+    <row r="21" ht="36" customHeight="1" spans="1:7">
       <c r="A21" s="10">
         <v>20</v>
       </c>
@@ -3124,25 +2969,22 @@
         <v>24</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>117</v>
+        <v>97</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>118</v>
+        <v>98</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="G21" s="8" t="s">
-        <v>120</v>
-      </c>
-      <c r="H21" s="17">
+        <v>99</v>
+      </c>
+      <c r="G21" s="17">
         <v>1</v>
       </c>
     </row>
-    <row r="22" ht="36" customHeight="1" spans="1:8">
+    <row r="22" ht="36" customHeight="1" spans="1:7">
       <c r="A22" s="6">
         <v>21</v>
       </c>
@@ -3150,100 +2992,65 @@
         <v>24</v>
       </c>
       <c r="C22" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="E22" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="D22" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>122</v>
-      </c>
       <c r="F22" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="G22" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="H22" s="16">
+        <v>102</v>
+      </c>
+      <c r="G22" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="23" ht="36" customHeight="1" spans="1:8">
+    <row r="23" ht="36" customHeight="1" spans="1:7">
       <c r="A23" s="10">
         <v>22</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>125</v>
+        <v>103</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>126</v>
+        <v>104</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>127</v>
+        <v>105</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>128</v>
+        <v>106</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>129</v>
-      </c>
-      <c r="G23" s="8" t="s">
-        <v>130</v>
-      </c>
-      <c r="H23" s="17">
+        <v>107</v>
+      </c>
+      <c r="G23" s="17">
         <v>4</v>
       </c>
     </row>
-    <row r="24" ht="36" customHeight="1" spans="1:8">
+    <row r="24" ht="36" customHeight="1" spans="1:7">
       <c r="A24" s="6">
         <v>23</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>125</v>
+        <v>103</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>126</v>
+        <v>104</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>131</v>
+        <v>108</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>128</v>
+        <v>109</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="G24" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="H24" s="16">
+        <v>110</v>
+      </c>
+      <c r="G24" s="16">
         <v>2</v>
-      </c>
-    </row>
-    <row r="25" ht="36" customHeight="1" spans="1:8">
-      <c r="A25" s="10">
-        <v>24</v>
-      </c>
-      <c r="B25" s="15" t="s">
-        <v>134</v>
-      </c>
-      <c r="C25" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="D25" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="E25" s="8" t="s">
-        <v>137</v>
-      </c>
-      <c r="F25" s="8" t="s">
-        <v>138</v>
-      </c>
-      <c r="G25" s="8" t="s">
-        <v>139</v>
-      </c>
-      <c r="H25" s="17">
-        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -3273,25 +3080,25 @@
         <v>30</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>140</v>
+        <v>111</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>141</v>
+        <v>112</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>142</v>
+        <v>113</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>143</v>
+        <v>114</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>144</v>
+        <v>115</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>145</v>
+        <v>116</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>146</v>
+        <v>117</v>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1" spans="1:8">
@@ -3299,25 +3106,25 @@
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>147</v>
+        <v>118</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>148</v>
+        <v>119</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>149</v>
+        <v>120</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>150</v>
+        <v>121</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>153</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3" ht="24" customHeight="1" spans="1:8">
@@ -3325,25 +3132,25 @@
         <v>2</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>154</v>
+        <v>125</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>155</v>
+        <v>126</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>156</v>
+        <v>127</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>157</v>
+        <v>128</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>158</v>
+        <v>129</v>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1" spans="1:8">
@@ -3351,25 +3158,25 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>159</v>
+        <v>130</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>160</v>
+        <v>131</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>161</v>
+        <v>132</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>162</v>
+        <v>133</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>163</v>
+        <v>134</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1" spans="1:8">
@@ -3377,25 +3184,25 @@
         <v>4</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>159</v>
+        <v>130</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>164</v>
+        <v>135</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>165</v>
+        <v>136</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>166</v>
+        <v>137</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>167</v>
+        <v>138</v>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1" spans="1:8">
@@ -3403,25 +3210,25 @@
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>159</v>
+        <v>130</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>168</v>
+        <v>139</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>169</v>
+        <v>140</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>166</v>
+        <v>137</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>170</v>
+        <v>141</v>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1" spans="1:8">
@@ -3429,25 +3236,25 @@
         <v>6</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>159</v>
+        <v>130</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>171</v>
+        <v>142</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>165</v>
+        <v>136</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>166</v>
+        <v>137</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>172</v>
+        <v>143</v>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1" spans="1:8">
@@ -3455,25 +3262,25 @@
         <v>7</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>159</v>
+        <v>130</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>173</v>
+        <v>144</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>174</v>
+        <v>145</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>166</v>
+        <v>137</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>175</v>
+        <v>146</v>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1" spans="1:8">
@@ -3481,25 +3288,25 @@
         <v>8</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>159</v>
+        <v>130</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>176</v>
+        <v>147</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>177</v>
+        <v>148</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>166</v>
+        <v>137</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>178</v>
+        <v>149</v>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1" spans="1:8">
@@ -3507,25 +3314,25 @@
         <v>9</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>159</v>
+        <v>130</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>179</v>
+        <v>150</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>165</v>
+        <v>136</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>166</v>
+        <v>137</v>
       </c>
       <c r="F10" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="H10" s="3" t="s">
         <v>151</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1" spans="1:8">
@@ -3533,25 +3340,25 @@
         <v>10</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>181</v>
+        <v>152</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>182</v>
+        <v>153</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>183</v>
+        <v>154</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>166</v>
+        <v>137</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>184</v>
+        <v>155</v>
       </c>
     </row>
     <row r="12" ht="24" customHeight="1" spans="1:8">
@@ -3559,25 +3366,25 @@
         <v>11</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>181</v>
+        <v>152</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>185</v>
+        <v>156</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>183</v>
+        <v>154</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>166</v>
+        <v>137</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>186</v>
+        <v>157</v>
       </c>
     </row>
     <row r="13" ht="24" customHeight="1" spans="1:8">
@@ -3585,25 +3392,25 @@
         <v>12</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>181</v>
+        <v>152</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>187</v>
+        <v>158</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>188</v>
+        <v>159</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>166</v>
+        <v>137</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>189</v>
+        <v>160</v>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1" spans="1:8">
@@ -3611,25 +3418,25 @@
         <v>13</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>181</v>
+        <v>152</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>190</v>
+        <v>161</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>191</v>
+        <v>162</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>166</v>
+        <v>137</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>192</v>
+        <v>163</v>
       </c>
     </row>
     <row r="15" ht="24" customHeight="1" spans="1:8">
@@ -3637,25 +3444,25 @@
         <v>14</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>181</v>
+        <v>152</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>193</v>
+        <v>164</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>169</v>
+        <v>140</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>166</v>
+        <v>137</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>194</v>
+        <v>165</v>
       </c>
     </row>
     <row r="16" ht="24" customHeight="1" spans="1:8">
@@ -3663,25 +3470,25 @@
         <v>15</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>181</v>
+        <v>152</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>195</v>
+        <v>166</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>177</v>
+        <v>148</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>166</v>
+        <v>137</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>196</v>
+        <v>167</v>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1" spans="1:8">
@@ -3689,25 +3496,25 @@
         <v>16</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>197</v>
+        <v>168</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>198</v>
+        <v>169</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>177</v>
+        <v>148</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>199</v>
+        <v>170</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>200</v>
+        <v>171</v>
       </c>
       <c r="H17" s="8" t="s">
-        <v>201</v>
+        <v>172</v>
       </c>
     </row>
     <row r="18" ht="24" customHeight="1" spans="1:8">
@@ -3715,25 +3522,25 @@
         <v>17</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>197</v>
+        <v>168</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>202</v>
+        <v>173</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>177</v>
+        <v>148</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>203</v>
+        <v>174</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>200</v>
+        <v>171</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>204</v>
+        <v>175</v>
       </c>
     </row>
     <row r="19" ht="24" customHeight="1" spans="1:8">
@@ -3741,25 +3548,25 @@
         <v>18</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>205</v>
+        <v>176</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>206</v>
+        <v>177</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>207</v>
+        <v>178</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>208</v>
+        <v>179</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H19" s="8" t="s">
-        <v>209</v>
+        <v>180</v>
       </c>
     </row>
     <row r="20" ht="24" customHeight="1" spans="1:8">
@@ -3767,25 +3574,25 @@
         <v>19</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>205</v>
+        <v>176</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>210</v>
+        <v>181</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>177</v>
+        <v>148</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>211</v>
+        <v>182</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>212</v>
+        <v>183</v>
       </c>
     </row>
     <row r="21" ht="24" customHeight="1" spans="1:8">
@@ -3793,25 +3600,25 @@
         <v>20</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>205</v>
+        <v>176</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>213</v>
+        <v>184</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>177</v>
+        <v>148</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>214</v>
+        <v>185</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H21" s="8" t="s">
-        <v>215</v>
+        <v>186</v>
       </c>
     </row>
     <row r="22" ht="24" customHeight="1" spans="1:8">
@@ -3819,25 +3626,25 @@
         <v>21</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>205</v>
+        <v>176</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>216</v>
+        <v>187</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>177</v>
+        <v>148</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>217</v>
+        <v>188</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>218</v>
+        <v>189</v>
       </c>
     </row>
     <row r="23" ht="24" customHeight="1" spans="1:8">
@@ -3845,25 +3652,25 @@
         <v>22</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>219</v>
+        <v>190</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>220</v>
+        <v>191</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>221</v>
+        <v>192</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>222</v>
+        <v>193</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>223</v>
+        <v>194</v>
       </c>
       <c r="H23" s="8" t="s">
-        <v>224</v>
+        <v>195</v>
       </c>
     </row>
   </sheetData>
@@ -3890,1094 +3697,1094 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:8">
       <c r="A1" s="1" t="s">
-        <v>225</v>
+        <v>196</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>226</v>
+        <v>197</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>227</v>
+        <v>198</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>228</v>
+        <v>199</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>229</v>
+        <v>200</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>230</v>
+        <v>201</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>231</v>
+        <v>202</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>232</v>
+        <v>203</v>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1" spans="1:8">
       <c r="A2" s="2" t="s">
-        <v>233</v>
+        <v>204</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>234</v>
+        <v>205</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>235</v>
+        <v>206</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>236</v>
+        <v>207</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>237</v>
+        <v>208</v>
       </c>
     </row>
     <row r="3" ht="24" customHeight="1" spans="1:8">
       <c r="A3" s="7" t="s">
-        <v>238</v>
+        <v>209</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>234</v>
+        <v>205</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>239</v>
+        <v>210</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>240</v>
+        <v>211</v>
       </c>
       <c r="G3" s="10" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>241</v>
+        <v>212</v>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1" spans="1:8">
       <c r="A4" s="2" t="s">
-        <v>242</v>
+        <v>213</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>243</v>
+        <v>214</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>244</v>
+        <v>215</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>245</v>
+        <v>216</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>246</v>
+        <v>217</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1" spans="1:8">
       <c r="A5" s="7" t="s">
-        <v>247</v>
+        <v>218</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>243</v>
+        <v>214</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>248</v>
+        <v>219</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>245</v>
+        <v>216</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>200</v>
+        <v>171</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>249</v>
+        <v>220</v>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1" spans="1:8">
       <c r="A6" s="2" t="s">
-        <v>250</v>
+        <v>221</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>243</v>
+        <v>214</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>251</v>
+        <v>222</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>245</v>
+        <v>216</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>200</v>
+        <v>171</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>252</v>
+        <v>223</v>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1" spans="1:8">
       <c r="A7" s="7" t="s">
-        <v>253</v>
+        <v>224</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>254</v>
+        <v>225</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>255</v>
+        <v>226</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>240</v>
+        <v>211</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>256</v>
+        <v>227</v>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1" spans="1:8">
       <c r="A8" s="2" t="s">
-        <v>257</v>
+        <v>228</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>254</v>
+        <v>225</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>258</v>
+        <v>229</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>259</v>
+        <v>230</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>260</v>
+        <v>231</v>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1" spans="1:8">
       <c r="A9" s="7" t="s">
-        <v>261</v>
+        <v>232</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>254</v>
+        <v>225</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>262</v>
+        <v>233</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>259</v>
+        <v>230</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>263</v>
+        <v>234</v>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1" spans="1:8">
       <c r="A10" s="2" t="s">
-        <v>264</v>
+        <v>235</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>254</v>
+        <v>225</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>265</v>
+        <v>236</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>259</v>
+        <v>230</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>266</v>
+        <v>237</v>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1" spans="1:8">
       <c r="A11" s="7" t="s">
-        <v>267</v>
+        <v>238</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>268</v>
+        <v>239</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>269</v>
+        <v>240</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>270</v>
+        <v>241</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>271</v>
+        <v>242</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>223</v>
+        <v>194</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>272</v>
+        <v>243</v>
       </c>
     </row>
     <row r="12" ht="24" customHeight="1" spans="1:8">
       <c r="A12" s="2" t="s">
-        <v>273</v>
+        <v>244</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>268</v>
+        <v>239</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>274</v>
+        <v>245</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>275</v>
+        <v>246</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>276</v>
+        <v>247</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>200</v>
+        <v>171</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>277</v>
+        <v>248</v>
       </c>
     </row>
     <row r="13" ht="24" customHeight="1" spans="1:8">
       <c r="A13" s="7" t="s">
-        <v>278</v>
+        <v>249</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>268</v>
+        <v>239</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>279</v>
+        <v>250</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>280</v>
+        <v>251</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>200</v>
+        <v>171</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>281</v>
+        <v>252</v>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1" spans="1:8">
       <c r="A14" s="2" t="s">
-        <v>282</v>
+        <v>253</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>268</v>
+        <v>239</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>274</v>
+        <v>245</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>279</v>
+        <v>250</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>283</v>
+        <v>254</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>200</v>
+        <v>171</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>284</v>
+        <v>255</v>
       </c>
     </row>
     <row r="15" ht="24" customHeight="1" spans="1:8">
       <c r="A15" s="7" t="s">
-        <v>285</v>
+        <v>256</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>268</v>
+        <v>239</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="D15" s="12" t="s">
-        <v>286</v>
+        <v>257</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>287</v>
+        <v>258</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>283</v>
+        <v>254</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>200</v>
+        <v>171</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>288</v>
+        <v>259</v>
       </c>
     </row>
     <row r="16" ht="24" customHeight="1" spans="1:8">
       <c r="A16" s="2" t="s">
-        <v>289</v>
+        <v>260</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>268</v>
+        <v>239</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>290</v>
+        <v>261</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>287</v>
+        <v>258</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>291</v>
+        <v>262</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>200</v>
+        <v>171</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>292</v>
+        <v>263</v>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1" spans="1:8">
       <c r="A17" s="7" t="s">
-        <v>293</v>
+        <v>264</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>268</v>
+        <v>239</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>294</v>
+        <v>265</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>280</v>
+        <v>251</v>
       </c>
       <c r="G17" s="10" t="s">
-        <v>223</v>
+        <v>194</v>
       </c>
       <c r="H17" s="8" t="s">
-        <v>295</v>
+        <v>266</v>
       </c>
     </row>
     <row r="18" ht="24" customHeight="1" spans="1:8">
       <c r="A18" s="2" t="s">
-        <v>296</v>
+        <v>267</v>
       </c>
       <c r="B18" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>257</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>265</v>
+      </c>
+      <c r="F18" s="3" t="s">
         <v>268</v>
       </c>
-      <c r="C18" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="D18" s="12" t="s">
-        <v>286</v>
-      </c>
-      <c r="E18" s="5" t="s">
-        <v>294</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>297</v>
-      </c>
       <c r="G18" s="6" t="s">
-        <v>200</v>
+        <v>171</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>298</v>
+        <v>269</v>
       </c>
     </row>
     <row r="19" ht="24" customHeight="1" spans="1:8">
       <c r="A19" s="7" t="s">
-        <v>299</v>
+        <v>270</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>268</v>
+        <v>239</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>300</v>
+        <v>271</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>280</v>
+        <v>251</v>
       </c>
       <c r="G19" s="10" t="s">
-        <v>223</v>
+        <v>194</v>
       </c>
       <c r="H19" s="8" t="s">
-        <v>301</v>
+        <v>272</v>
       </c>
     </row>
     <row r="20" ht="24" customHeight="1" spans="1:8">
       <c r="A20" s="2" t="s">
-        <v>302</v>
+        <v>273</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>268</v>
+        <v>239</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="D20" s="11" t="s">
+        <v>245</v>
+      </c>
+      <c r="E20" s="5" t="s">
         <v>274</v>
       </c>
-      <c r="E20" s="5" t="s">
-        <v>303</v>
-      </c>
       <c r="F20" s="3" t="s">
-        <v>304</v>
+        <v>275</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>200</v>
+        <v>171</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>305</v>
+        <v>276</v>
       </c>
     </row>
     <row r="21" ht="24" customHeight="1" spans="1:8">
       <c r="A21" s="7" t="s">
-        <v>306</v>
+        <v>277</v>
       </c>
       <c r="B21" s="8" t="s">
         <v>22</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>307</v>
+        <v>278</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>245</v>
+        <v>216</v>
       </c>
       <c r="G21" s="10" t="s">
-        <v>308</v>
+        <v>279</v>
       </c>
       <c r="H21" s="8" t="s">
-        <v>309</v>
+        <v>280</v>
       </c>
     </row>
     <row r="22" ht="24" customHeight="1" spans="1:8">
       <c r="A22" s="2" t="s">
-        <v>310</v>
+        <v>281</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>274</v>
+        <v>245</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>311</v>
+        <v>282</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>312</v>
+        <v>283</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>200</v>
+        <v>171</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>313</v>
+        <v>284</v>
       </c>
     </row>
     <row r="23" ht="24" customHeight="1" spans="1:8">
       <c r="A23" s="7" t="s">
-        <v>314</v>
+        <v>285</v>
       </c>
       <c r="B23" s="8" t="s">
         <v>22</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>315</v>
+        <v>286</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>316</v>
+        <v>287</v>
       </c>
       <c r="G23" s="10" t="s">
-        <v>200</v>
+        <v>171</v>
       </c>
       <c r="H23" s="8" t="s">
-        <v>317</v>
+        <v>288</v>
       </c>
     </row>
     <row r="24" ht="24" customHeight="1" spans="1:8">
       <c r="A24" s="2" t="s">
-        <v>318</v>
+        <v>289</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>81</v>
+        <v>70</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>319</v>
+        <v>290</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>320</v>
+        <v>291</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>321</v>
+        <v>292</v>
       </c>
     </row>
     <row r="25" ht="24" customHeight="1" spans="1:8">
       <c r="A25" s="7" t="s">
-        <v>322</v>
+        <v>293</v>
       </c>
       <c r="B25" s="8" t="s">
         <v>22</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>81</v>
+        <v>70</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>323</v>
+        <v>294</v>
       </c>
       <c r="F25" s="8" t="s">
-        <v>324</v>
+        <v>295</v>
       </c>
       <c r="G25" s="10" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H25" s="8" t="s">
-        <v>325</v>
+        <v>296</v>
       </c>
     </row>
     <row r="26" ht="24" customHeight="1" spans="1:8">
       <c r="A26" s="2" t="s">
-        <v>326</v>
+        <v>297</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>85</v>
+        <v>73</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>327</v>
+        <v>298</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>328</v>
+        <v>299</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>223</v>
+        <v>194</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>329</v>
+        <v>300</v>
       </c>
     </row>
     <row r="27" ht="24" customHeight="1" spans="1:8">
       <c r="A27" s="7" t="s">
-        <v>330</v>
+        <v>301</v>
       </c>
       <c r="B27" s="8" t="s">
         <v>22</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>85</v>
+        <v>73</v>
       </c>
       <c r="D27" s="11" t="s">
-        <v>274</v>
+        <v>245</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>331</v>
+        <v>302</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>332</v>
+        <v>303</v>
       </c>
       <c r="G27" s="10" t="s">
-        <v>200</v>
+        <v>171</v>
       </c>
       <c r="H27" s="8" t="s">
-        <v>333</v>
+        <v>304</v>
       </c>
     </row>
     <row r="28" ht="24" customHeight="1" spans="1:8">
       <c r="A28" s="2" t="s">
-        <v>334</v>
+        <v>305</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>335</v>
+        <v>306</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>336</v>
+        <v>307</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>337</v>
+        <v>308</v>
       </c>
     </row>
     <row r="29" ht="24" customHeight="1" spans="1:8">
       <c r="A29" s="7" t="s">
-        <v>338</v>
+        <v>309</v>
       </c>
       <c r="B29" s="8" t="s">
         <v>22</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>339</v>
+        <v>310</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>336</v>
+        <v>307</v>
       </c>
       <c r="G29" s="10" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H29" s="8" t="s">
-        <v>340</v>
+        <v>311</v>
       </c>
     </row>
     <row r="30" ht="24" customHeight="1" spans="1:8">
       <c r="A30" s="2" t="s">
-        <v>341</v>
+        <v>312</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>342</v>
+        <v>313</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>336</v>
+        <v>307</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>343</v>
+        <v>314</v>
       </c>
     </row>
     <row r="31" ht="24" customHeight="1" spans="1:8">
       <c r="A31" s="7" t="s">
-        <v>344</v>
+        <v>315</v>
       </c>
       <c r="B31" s="8" t="s">
         <v>22</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>345</v>
+        <v>316</v>
       </c>
       <c r="F31" s="8" t="s">
-        <v>336</v>
+        <v>307</v>
       </c>
       <c r="G31" s="10" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H31" s="8" t="s">
-        <v>346</v>
+        <v>317</v>
       </c>
     </row>
     <row r="32" ht="24" customHeight="1" spans="1:8">
       <c r="A32" s="2" t="s">
-        <v>347</v>
+        <v>318</v>
       </c>
       <c r="B32" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>348</v>
+        <v>319</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>336</v>
+        <v>307</v>
       </c>
       <c r="G32" s="6" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H32" s="3" t="s">
-        <v>349</v>
+        <v>320</v>
       </c>
     </row>
     <row r="33" ht="24" customHeight="1" spans="1:8">
       <c r="A33" s="7" t="s">
-        <v>350</v>
+        <v>321</v>
       </c>
       <c r="B33" s="8" t="s">
         <v>22</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>93</v>
+        <v>79</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>351</v>
+        <v>322</v>
       </c>
       <c r="F33" s="8" t="s">
-        <v>352</v>
+        <v>323</v>
       </c>
       <c r="G33" s="10" t="s">
-        <v>200</v>
+        <v>171</v>
       </c>
       <c r="H33" s="8" t="s">
-        <v>353</v>
+        <v>324</v>
       </c>
     </row>
     <row r="34" ht="24" customHeight="1" spans="1:8">
       <c r="A34" s="2" t="s">
-        <v>354</v>
+        <v>325</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>24</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>355</v>
+        <v>326</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>259</v>
+        <v>230</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H34" s="3" t="s">
-        <v>356</v>
+        <v>327</v>
       </c>
     </row>
     <row r="35" ht="24" customHeight="1" spans="1:8">
       <c r="A35" s="7" t="s">
-        <v>357</v>
+        <v>328</v>
       </c>
       <c r="B35" s="8" t="s">
         <v>24</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="E35" s="9" t="s">
-        <v>358</v>
+        <v>329</v>
       </c>
       <c r="F35" s="8" t="s">
-        <v>259</v>
+        <v>230</v>
       </c>
       <c r="G35" s="10" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H35" s="8" t="s">
-        <v>359</v>
+        <v>330</v>
       </c>
     </row>
     <row r="36" ht="24" customHeight="1" spans="1:8">
       <c r="A36" s="2" t="s">
-        <v>360</v>
+        <v>331</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>24</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>105</v>
+        <v>88</v>
       </c>
       <c r="D36" s="11" t="s">
-        <v>274</v>
+        <v>245</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>361</v>
+        <v>332</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>362</v>
+        <v>333</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H36" s="3" t="s">
-        <v>363</v>
+        <v>334</v>
       </c>
     </row>
     <row r="37" ht="24" customHeight="1" spans="1:8">
       <c r="A37" s="7" t="s">
-        <v>364</v>
+        <v>335</v>
       </c>
       <c r="B37" s="8" t="s">
         <v>24</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>105</v>
+        <v>88</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>365</v>
+        <v>336</v>
       </c>
       <c r="F37" s="8" t="s">
-        <v>259</v>
+        <v>230</v>
       </c>
       <c r="G37" s="10" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H37" s="8" t="s">
-        <v>366</v>
+        <v>337</v>
       </c>
     </row>
     <row r="38" ht="24" customHeight="1" spans="1:8">
       <c r="A38" s="2" t="s">
-        <v>367</v>
+        <v>338</v>
       </c>
       <c r="B38" s="3" t="s">
         <v>24</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>105</v>
+        <v>88</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>368</v>
+        <v>339</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>369</v>
+        <v>340</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H38" s="3" t="s">
-        <v>370</v>
+        <v>341</v>
       </c>
     </row>
     <row r="39" ht="24" customHeight="1" spans="1:8">
       <c r="A39" s="7" t="s">
-        <v>371</v>
+        <v>342</v>
       </c>
       <c r="B39" s="8" t="s">
         <v>24</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>372</v>
+        <v>343</v>
       </c>
       <c r="F39" s="8" t="s">
-        <v>259</v>
+        <v>230</v>
       </c>
       <c r="G39" s="10" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H39" s="8" t="s">
-        <v>373</v>
+        <v>344</v>
       </c>
     </row>
     <row r="40" ht="24" customHeight="1" spans="1:8">
       <c r="A40" s="2" t="s">
-        <v>374</v>
+        <v>345</v>
       </c>
       <c r="B40" s="3" t="s">
         <v>24</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>117</v>
+        <v>97</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>375</v>
+        <v>346</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>259</v>
+        <v>230</v>
       </c>
       <c r="G40" s="6" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H40" s="3" t="s">
-        <v>376</v>
+        <v>347</v>
       </c>
     </row>
     <row r="41" ht="24" customHeight="1" spans="1:8">
       <c r="A41" s="7" t="s">
-        <v>377</v>
+        <v>348</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>125</v>
+        <v>103</v>
       </c>
       <c r="C41" s="8" t="s">
-        <v>378</v>
+        <v>349</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>379</v>
+        <v>350</v>
       </c>
       <c r="F41" s="8" t="s">
-        <v>352</v>
+        <v>323</v>
       </c>
       <c r="G41" s="10" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H41" s="8" t="s">
-        <v>380</v>
+        <v>351</v>
       </c>
     </row>
     <row r="42" ht="24" customHeight="1" spans="1:8">
       <c r="A42" s="2" t="s">
-        <v>381</v>
+        <v>352</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>125</v>
+        <v>103</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>131</v>
+        <v>108</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>382</v>
+        <v>353</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>383</v>
+        <v>354</v>
       </c>
       <c r="G42" s="6" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
       <c r="H42" s="3" t="s">
-        <v>384</v>
+        <v>355</v>
       </c>
     </row>
   </sheetData>

</xml_diff>